<commit_message>
Auto‑update: 2026-10-08 03:29:20 UTC
</commit_message>
<xml_diff>
--- a/resources/bad_words.xlsx
+++ b/resources/bad_words.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C209"/>
+  <dimension ref="A1:C213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1474,24 +1474,24 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Xaromi</t>
+          <t>Totaq</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>143</v>
+        <v>64</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Ya yebal tebya</t>
+          <t>Xaromi</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -1500,11 +1500,11 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>233</v>
+        <v>143</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Yban</t>
+          <t>Ya yebal tebya</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -1513,11 +1513,11 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>198</v>
+        <v>233</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Ybat</t>
+          <t>Yban</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -1526,11 +1526,11 @@
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>15</v>
+        <v>198</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Yeban</t>
+          <t>Ybat</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -1539,11 +1539,11 @@
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>62</v>
+        <v>15</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Yebanutiy</t>
+          <t>Yeban</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -1552,63 +1552,63 @@
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>373</v>
+        <v>62</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Yebat</t>
+          <t>Yebanutiy</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>83</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>2</v>
+        <v>373</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Yiban</t>
+          <t>Yebat</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1</v>
+        <v>83</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>372</v>
+        <v>2</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Yobbana</t>
+          <t>Yiban</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>183</v>
+        <v>372</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Zaybal</t>
+          <t>Yobbana</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>78</v>
+        <v>183</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>ahmoq</t>
+          <t>Zaybal</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -1617,11 +1617,11 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>142</v>
+        <v>78</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ahuel</t>
+          <t>ahmoq</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -1630,11 +1630,11 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>22</v>
+        <v>142</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>am</t>
+          <t>ahuel</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -1643,37 +1643,37 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>329</v>
+        <v>22</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>ambaliq</t>
+          <t>am</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>223</v>
+        <v>329</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>amcha</t>
+          <t>ambaliq</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>108</v>
+        <v>223</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>aminga</t>
+          <t>amcha</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -1682,89 +1682,89 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>349</v>
+        <v>108</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>amingga ske</t>
+          <t>aminga</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>97</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>16</v>
+        <v>349</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>ammisan</t>
+          <t>amingga ske</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>360</v>
+        <v>16</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>axmoq</t>
+          <t>ammisan</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>50</v>
+        <v>93</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>236</v>
+        <v>360</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>basharenga qotogm</t>
+          <t>axmoq</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>330</v>
+        <v>236</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>bich</t>
+          <t>basharenga qotogm</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>93</v>
+        <v>330</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>bitch</t>
+          <t>bich</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>ble</t>
+          <t>bitch</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -1773,11 +1773,11 @@
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>53</v>
+        <v>99</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>blet</t>
+          <t>ble</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -1786,37 +1786,37 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>blyat</t>
+          <t>blet</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>261</v>
+        <v>30</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>bo'qidish</t>
+          <t>blyat</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>bo'qkalla</t>
+          <t>bo'qidish</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -1825,11 +1825,11 @@
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>244</v>
+        <v>262</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>boq</t>
+          <t>bo'qkalla</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -1838,24 +1838,24 @@
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>9</v>
+        <v>244</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>buvini ami</t>
+          <t>boq</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>buvini amiga ske</t>
+          <t>buvini ami</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -1864,37 +1864,37 @@
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>279</v>
+        <v>10</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>chmo</t>
+          <t>buvini amiga ske</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>368</v>
+        <v>38</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>cho'choq</t>
+          <t>chichqoq</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>50</v>
+        <v>76</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>chumo</t>
+          <t>chmo</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -1903,37 +1903,37 @@
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>305</v>
+        <v>368</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>dabba</t>
+          <t>cho'choq</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>370</v>
+        <v>280</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>dalban</t>
+          <t>chumo</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>107</v>
+        <v>305</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>dalbayob</t>
+          <t>dabba</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -1942,24 +1942,24 @@
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>278</v>
+        <v>370</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>daun</t>
+          <t>dalban</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>84</v>
+        <v>107</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>dinnaxuy</t>
+          <t>dalbayob</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -1968,24 +1968,24 @@
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>8</v>
+        <v>278</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>foxisha qanchiq</t>
+          <t>daun</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>79</v>
+        <v>1</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>110</v>
+        <v>84</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>fuck</t>
+          <t>dinnaxuy</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -1994,24 +1994,24 @@
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>324</v>
+        <v>8</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>fuck off</t>
+          <t>foxisha qanchiq</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>fucking</t>
+          <t>fuck</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -2020,37 +2020,37 @@
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>160</v>
+        <v>324</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>gandon</t>
+          <t>fuck off</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1</v>
+        <v>75</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>361</v>
+        <v>111</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>garang</t>
+          <t>fucking</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>gay</t>
+          <t>gandon</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -2059,24 +2059,24 @@
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>166</v>
+        <v>361</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>gey</t>
+          <t>garang</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>gnida</t>
+          <t>gay</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -2085,11 +2085,11 @@
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>227</v>
+        <v>166</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>haromi</t>
+          <t>gey</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -2098,11 +2098,11 @@
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>203</v>
+        <v>161</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>hunasa</t>
+          <t>gnida</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -2111,89 +2111,89 @@
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>334</v>
+        <v>227</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>idi naxuy</t>
+          <t>haromi</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>90</v>
+        <v>1</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>357</v>
+        <v>203</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>iflos</t>
+          <t>hunasa</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>48</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>idi naxuy</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>260</v>
+        <v>357</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>itbet</t>
+          <t>iflos</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>1</v>
+        <v>48</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>95</v>
+        <v>46</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>jala</t>
+          <t>iprisqi</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>98</v>
+        <v>331</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>jala ble</t>
+          <t>it</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>303</v>
+        <v>260</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>jalaaap</t>
+          <t>itbet</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -2202,11 +2202,11 @@
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>jalab</t>
+          <t>jala</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -2215,11 +2215,11 @@
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>158</v>
+        <v>98</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>jalap</t>
+          <t>jala ble</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -2228,11 +2228,11 @@
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>88</v>
+        <v>303</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>jalla</t>
+          <t>jalaaap</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -2241,11 +2241,11 @@
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>jallap</t>
+          <t>jalab</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -2254,102 +2254,102 @@
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>374</v>
+        <v>158</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>jentra miyya</t>
+          <t>jalap</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>24</v>
+        <v>88</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>jinni</t>
+          <t>jalla</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>366</v>
+        <v>89</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>kashanda</t>
+          <t>jallap</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>33</v>
+        <v>374</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>ko't</t>
+          <t>jentra miyya</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>kot</t>
+          <t>jinni</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>310</v>
+        <v>366</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>lox</t>
+          <t>kashanda</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>293</v>
+        <v>33</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>mol</t>
+          <t>ko't</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>306</v>
+        <v>26</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>nedagon</t>
+          <t>kot</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -2358,37 +2358,37 @@
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>199</v>
+        <v>310</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>nigga</t>
+          <t>lox</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>1</v>
+        <v>40</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>83</v>
+        <v>293</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>nigger</t>
+          <t>mol</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>23</v>
+        <v>306</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>om</t>
+          <t>nedagon</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -2397,11 +2397,11 @@
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>96</v>
+        <v>199</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>onangni</t>
+          <t>nigga</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -2410,63 +2410,63 @@
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>327</v>
+        <v>83</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>onangni ami</t>
+          <t>nigger</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>341</v>
+        <v>23</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>onangni sikay</t>
+          <t>om</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>365</v>
+        <v>96</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>oneni ami</t>
+          <t>onangni</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>184</v>
+        <v>327</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>oom</t>
+          <t>onangni ami</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>363</v>
+        <v>341</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>oʻl</t>
+          <t>onangni sikay</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -2475,50 +2475,50 @@
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>12</v>
+        <v>365</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>p1zdes</t>
+          <t>oneni ami</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>333</v>
+        <v>184</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>pashol na xuy</t>
+          <t>oom</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>75</v>
+        <v>363</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>pidaras</t>
+          <t>oʻl</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>74</v>
+        <v>12</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>pidaraz</t>
+          <t>p1zdes</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -2527,24 +2527,24 @@
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>97</v>
+        <v>333</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>pidr</t>
+          <t>pashol na xuy</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>pizda</t>
+          <t>pidaras</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -2553,11 +2553,11 @@
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>11</v>
+        <v>74</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>pizdes</t>
+          <t>pidaraz</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -2566,11 +2566,11 @@
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>qanjiq</t>
+          <t>pidr</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -2579,24 +2579,24 @@
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>36</v>
+        <v>86</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>qanju</t>
+          <t>pizda</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>qo'toq</t>
+          <t>pizdes</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -2605,11 +2605,11 @@
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>28</v>
+        <v>92</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>qo'toqbosh</t>
+          <t>qanjiq</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -2618,24 +2618,24 @@
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>116</v>
+        <v>36</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>qotaq</t>
+          <t>qanju</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>234</v>
+        <v>85</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>qoto</t>
+          <t>qo'toq</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -2644,11 +2644,11 @@
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>72</v>
+        <v>28</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>qotoq</t>
+          <t>qo'toqbosh</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -2657,11 +2657,11 @@
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>282</v>
+        <v>116</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>qutoq</t>
+          <t>qotaq</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -2670,11 +2670,11 @@
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>31</v>
+        <v>234</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>seks</t>
+          <t>qoto</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -2683,11 +2683,11 @@
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>seksi baby</t>
+          <t>qotoq</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -2696,11 +2696,11 @@
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>13</v>
+        <v>282</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>sex</t>
+          <t>qutoq</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -2709,37 +2709,37 @@
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>348</v>
+        <v>31</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>sexy woman</t>
+          <t>seks</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>322</v>
+        <v>71</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>shavqatsiz</t>
+          <t>seksi baby</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>109</v>
+        <v>13</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>sikay</t>
+          <t>sex</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -2748,37 +2748,37 @@
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>134</v>
+        <v>348</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>sike</t>
+          <t>sexy woman</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>1</v>
+        <v>75</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>18</v>
+        <v>322</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>sikish</t>
+          <t>shavqatsiz</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>20</v>
+        <v>109</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>siktim</t>
+          <t>sikay</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -2787,11 +2787,11 @@
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>17</v>
+        <v>134</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>sikvoti</t>
+          <t>sike</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -2800,11 +2800,11 @@
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>73</v>
+        <v>18</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>skay</t>
+          <t>sikish</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -2813,11 +2813,11 @@
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>ske</t>
+          <t>siktim</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -2826,11 +2826,11 @@
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>159</v>
+        <v>17</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>skey</t>
+          <t>sikvoti</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -2839,11 +2839,11 @@
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>106</v>
+        <v>73</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>suchka</t>
+          <t>skay</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -2852,11 +2852,11 @@
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>suka</t>
+          <t>ske</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -2865,11 +2865,11 @@
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>119</v>
+        <v>159</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>sukka</t>
+          <t>skey</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -2878,11 +2878,11 @@
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>tashsho</t>
+          <t>suchka</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -2891,11 +2891,11 @@
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>32</v>
+        <v>90</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>tupoy</t>
+          <t>suka</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -2904,11 +2904,11 @@
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>162</v>
+        <v>119</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>tvar</t>
+          <t>sukka</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -2917,11 +2917,11 @@
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>163</v>
+        <v>87</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>tvariddin</t>
+          <t>tashsho</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -2930,11 +2930,11 @@
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>137</v>
+        <v>32</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>wtf</t>
+          <t>tupoy</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -2943,11 +2943,11 @@
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>27</v>
+        <v>162</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>xaromi</t>
+          <t>tvar</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -2956,11 +2956,11 @@
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>140</v>
+        <v>163</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>xuyeplet</t>
+          <t>tvariddin</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -2969,11 +2969,11 @@
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>xuyesos</t>
+          <t>wtf</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -2982,11 +2982,11 @@
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>xuyila</t>
+          <t>xaromi</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -2995,11 +2995,11 @@
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>19</v>
+        <v>140</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>yban</t>
+          <t>xuyeplet</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -3008,11 +3008,11 @@
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>281</v>
+        <v>139</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>yeban</t>
+          <t>xuyesos</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -3021,11 +3021,11 @@
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>yebanashka</t>
+          <t>xuyila</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -3034,11 +3034,11 @@
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>287</v>
+        <v>19</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>yebat</t>
+          <t>yban</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -3047,11 +3047,11 @@
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>91</v>
+        <v>281</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>yebbat</t>
+          <t>yeban</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -3060,24 +3060,24 @@
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>364</v>
+        <v>148</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>yeblan</t>
+          <t>yebanashka</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>44</v>
+        <v>1</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>145</v>
+        <v>287</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>yebnu</t>
+          <t>yebat</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -3086,11 +3086,11 @@
     </row>
     <row r="205">
       <c r="A205" t="n">
-        <v>144</v>
+        <v>91</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>yebu</t>
+          <t>yebbat</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -3099,24 +3099,24 @@
     </row>
     <row r="206">
       <c r="A206" t="n">
-        <v>14</v>
+        <v>364</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>yetim</t>
+          <t>yeblan</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>1</v>
+        <v>44</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
-        <v>94</v>
+        <v>145</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>yetm</t>
+          <t>yebnu</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -3125,11 +3125,11 @@
     </row>
     <row r="208">
       <c r="A208" t="n">
-        <v>277</v>
+        <v>144</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>yiban</t>
+          <t>yebu</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -3138,14 +3138,66 @@
     </row>
     <row r="209">
       <c r="A209" t="n">
+        <v>14</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>yetim</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>94</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>yetm</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>277</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>yiban</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>44</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>yiban dalbayob</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
         <v>283</v>
       </c>
-      <c r="B209" t="inlineStr">
+      <c r="B213" t="inlineStr">
         <is>
           <t>yibanat</t>
         </is>
       </c>
-      <c r="C209" t="n">
+      <c r="C213" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>